<commit_message>
v6: exclude 371 species with IUCN ranges outside US EEZ; fix missing mammal range maps
- Exclude 371 species (343 fish, 20 invertebrates, 6 corals, 2 mammals)
  whose IUCN expert range maps fall entirely outside the US EEZ. Their
  AquaMaps predictions in US waters were edge-of-range artifacts with
  near-zero suitability. Valid species: 9,819 → 9,424.
- Ingest 3 missing mammal IUCN ranges (Phoca vitulina, Trichechus manatus,
  Pusa hispida) from newer MAMMALS.zip download.
- Fix merge cleanup bug: delete stale merged models before the zero-cells
  check, not after.
- Resolves all 12 SEFSC-flagged marine mammals in Gulf of America.
- Score impact negligible across all Program Areas.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/msens-summary_programareas_v4b/table_programarea_scores_v4b.xlsx
+++ b/figs/msens-summary_programareas_v4b/table_programarea_scores_v4b.xlsx
@@ -47,18 +47,18 @@
     <t xml:space="preserve">Area (1,000 km2)</t>
   </si>
   <si>
+    <t xml:space="preserve">Cook Inlet (COK)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hope Basin (HOP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cook Inlet (COK)</t>
+    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
   </si>
   <si>
     <t xml:space="preserve">St. George Basin (GEO)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
-  </si>
-  <si>
     <t xml:space="preserve">GOA Program Area A (GAA)</t>
   </si>
   <si>
@@ -68,10 +68,10 @@
     <t xml:space="preserve">Shumagin (SHU)</t>
   </si>
   <si>
+    <t xml:space="preserve">Southern California (SOC)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aleutian Arc (ALA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern California (SOC)</t>
   </si>
   <si>
     <t xml:space="preserve">Norton Basin (NOR)</t>
@@ -476,29 +476,31 @@
         <v>53</v>
       </c>
       <c r="C2" t="n">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="D2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E2" t="n">
         <v>70</v>
       </c>
       <c r="F2" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="G2" t="n">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="H2" t="n">
-        <v>33</v>
-      </c>
-      <c r="I2"/>
+        <v>41</v>
+      </c>
+      <c r="I2" t="n">
+        <v>49</v>
+      </c>
       <c r="J2" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="K2" t="n">
-        <v>52</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -506,34 +508,32 @@
         <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C3" t="n">
-        <v>99</v>
+        <v>39</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="E3" t="n">
         <v>70</v>
       </c>
       <c r="F3" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="G3" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="H3" t="n">
-        <v>41</v>
-      </c>
-      <c r="I3" t="n">
-        <v>49</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="I3"/>
       <c r="J3" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K3" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
@@ -541,34 +541,34 @@
         <v>13</v>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="D4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F4" t="n">
         <v>27</v>
       </c>
-      <c r="E4" t="n">
-        <v>37</v>
-      </c>
-      <c r="F4" t="n">
-        <v>32</v>
-      </c>
       <c r="G4" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="H4" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="I4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="J4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>283</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5">
@@ -576,34 +576,34 @@
         <v>14</v>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D5" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="F5" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G5" t="n">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="H5" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K5" t="n">
-        <v>383</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6">
@@ -626,7 +626,7 @@
         <v>32</v>
       </c>
       <c r="G6" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H6" t="n">
         <v>26</v>
@@ -719,31 +719,31 @@
         <v>30</v>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D9" t="n">
         <v>15</v>
       </c>
       <c r="E9" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F9" t="n">
+        <v>18</v>
+      </c>
+      <c r="G9" t="n">
+        <v>64</v>
+      </c>
+      <c r="H9" t="n">
         <v>15</v>
       </c>
-      <c r="G9" t="n">
-        <v>43</v>
-      </c>
-      <c r="H9" t="n">
-        <v>18</v>
-      </c>
       <c r="I9" t="n">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K9" t="n">
-        <v>870</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10">
@@ -754,31 +754,31 @@
         <v>29</v>
       </c>
       <c r="C10" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D10" t="n">
         <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F10" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" t="n">
+        <v>43</v>
+      </c>
+      <c r="H10" t="n">
         <v>18</v>
       </c>
-      <c r="G10" t="n">
-        <v>64</v>
-      </c>
-      <c r="H10" t="n">
-        <v>15</v>
-      </c>
       <c r="I10" t="n">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="J10" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>276</v>
+        <v>870</v>
       </c>
     </row>
     <row r="11">
@@ -786,7 +786,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" t="n">
         <v>92</v>
@@ -801,7 +801,7 @@
         <v>12</v>
       </c>
       <c r="G11" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H11" t="n">
         <v>7</v>
@@ -834,7 +834,7 @@
         <v>14</v>
       </c>
       <c r="G12" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H12" t="n">
         <v>17</v>
@@ -920,7 +920,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" t="n">
         <v>79</v>
@@ -935,7 +935,7 @@
         <v>12</v>
       </c>
       <c r="G15" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H15" t="n">
         <v>8</v>
@@ -1003,7 +1003,7 @@
         <v>8</v>
       </c>
       <c r="G17" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H17" t="n">
         <v>8</v>
@@ -1023,7 +1023,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18" t="n">
         <v>37</v>
@@ -1038,7 +1038,7 @@
         <v>6</v>
       </c>
       <c r="G18" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H18" t="n">
         <v>10</v>
@@ -1056,7 +1056,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C19" t="n">
         <v>5</v>
@@ -1071,7 +1071,7 @@
         <v>18</v>
       </c>
       <c r="G19" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H19" t="n">
         <v>21</v>
@@ -1104,7 +1104,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H20" t="n">
         <v>5</v>
@@ -1122,7 +1122,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>

</xml_diff>